<commit_message>
Hide removed doctors from site
</commit_message>
<xml_diff>
--- a/yandex-doctors-feed/biorise-doctors-feed.xlsx
+++ b/yandex-doctors-feed/biorise-doctors-feed.xlsx
@@ -1397,7 +1397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="24.5" customWidth="1" style="6" min="1" max="1"/>
@@ -1466,41 +1466,23 @@
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>base_boboeva</t>
+          <t>base_gaylis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>Первичный приём эндокринолога</t>
+          <t>Первичный приём диетолога</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr"/>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Первичный приём эндокринолога</t>
+          <t>Первичный приём диетолога</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>base_gaylis</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Первичный приём диетолога</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr"/>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Первичный приём диетолога</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
         <is>
           <t>base_tregubova</t>
         </is>
@@ -1858,17 +1840,17 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Бобоева Наталья</t>
+          <t>Гайлис Алёна Алексеевна</t>
         </is>
       </c>
       <c r="B3" s="14" t="inlineStr">
         <is>
-          <t>boboeva</t>
+          <t>gaylis</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/vrachi/boboeva/</t>
+          <t>https://biorise-clinic.ru/vrachi/gaylis/</t>
         </is>
       </c>
       <c r="D3" s="17" t="n">
@@ -1888,12 +1870,12 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/vrachi/boboeva/</t>
+          <t>https://biorise-clinic.ru/vrachi/gaylis/</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Врач-эндокринолог. Работает с хроническими эндокринными заболеваниями.</t>
+          <t>Врач-эндокринолог. Основные направления: ожирение, гипотиреоз, сахарный диабет, НАЖБП, железодефицитная анемия.</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
@@ -1903,7 +1885,7 @@
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/optimized/doctors/boboeva.webp</t>
+          <t>https://biorise-clinic.ru/optimized/doctors/gaylis-2.webp</t>
         </is>
       </c>
       <c r="M3" s="7" t="inlineStr"/>
@@ -1959,34 +1941,34 @@
       </c>
       <c r="AB3" s="6" t="inlineStr">
         <is>
-          <t>boboeva</t>
+          <t>gaylis</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Гайлис Алёна Алексеевна</t>
+          <t>Трегубова Лиана Игоревна</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t>gaylis</t>
+          <t>tregubova</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/vrachi/gaylis/</t>
+          <t>https://biorise-clinic.ru/vrachi/tregubova/</t>
         </is>
       </c>
       <c r="D4" s="17" t="n">
-        <v>2800</v>
+        <v>2200</v>
       </c>
       <c r="E4" s="17" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" s="6" t="inlineStr">
         <is>
-          <t>Первичный приём эндокринолога</t>
+          <t>Первичный приём диетолога</t>
         </is>
       </c>
       <c r="H4" s="6" t="inlineStr">
@@ -1996,22 +1978,22 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/vrachi/gaylis/</t>
+          <t>https://biorise-clinic.ru/vrachi/tregubova/</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Врач-эндокринолог. Основные направления: ожирение, гипотиреоз, сахарный диабет, НАЖБП, железодефицитная анемия.</t>
+          <t>Врач-диетолог, специализируется на интегративной превентивной и антивозрастной медицине.</t>
         </is>
       </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
-          <t>эндокринолог</t>
+          <t>диетолог</t>
         </is>
       </c>
       <c r="L4" s="6" t="inlineStr">
         <is>
-          <t>https://biorise-clinic.ru/optimized/doctors/gaylis-2.webp</t>
+          <t>https://biorise-clinic.ru/optimized/doctors/tregubova.webp</t>
         </is>
       </c>
       <c r="M4" s="7" t="inlineStr"/>
@@ -2067,117 +2049,14 @@
       </c>
       <c r="AB4" s="6" t="inlineStr">
         <is>
-          <t>gaylis</t>
+          <t>tregubova</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Трегубова Лиана Игоревна</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>tregubova</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>https://biorise-clinic.ru/vrachi/tregubova/</t>
-        </is>
-      </c>
-      <c r="D5" s="17" t="n">
-        <v>2200</v>
-      </c>
-      <c r="E5" s="17" t="inlineStr"/>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Первичный приём диетолога</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Да</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>https://biorise-clinic.ru/vrachi/tregubova/</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>Врач-диетолог, специализируется на интегративной превентивной и антивозрастной медицине.</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>диетолог</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>https://biorise-clinic.ru/optimized/doctors/tregubova.webp</t>
-        </is>
-      </c>
-      <c r="M5" s="7" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>clinic_dybenko</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr"/>
-      <c r="P5" t="inlineStr"/>
-      <c r="Q5" t="inlineStr"/>
-      <c r="R5" t="inlineStr"/>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>ИСТИНА</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>ЛОЖЬ</t>
-        </is>
-      </c>
-      <c r="V5" t="inlineStr">
-        <is>
-          <t>8 996 749 97 47</t>
-        </is>
-      </c>
-      <c r="W5" t="inlineStr">
-        <is>
-          <t>ЛОЖЬ</t>
-        </is>
-      </c>
-      <c r="X5" t="inlineStr">
-        <is>
-          <t>ЛОЖЬ</t>
-        </is>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>ЛОЖЬ</t>
-        </is>
-      </c>
-      <c r="Z5" t="inlineStr">
-        <is>
-          <t>ИСТИНА</t>
-        </is>
-      </c>
-      <c r="AA5" t="inlineStr">
-        <is>
-          <t>ЛОЖЬ</t>
-        </is>
-      </c>
-      <c r="AB5" t="inlineStr">
-        <is>
-          <t>tregubova</t>
-        </is>
-      </c>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="M5" s="7" t="n"/>
     </row>
     <row r="6">
       <c r="D6" s="17" t="n"/>

</xml_diff>